<commit_message>
romania-deficit: glosar si abrevieri, termeni explicati la prima aparitie
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/romania-deficit/Model_DSA_Romania.xlsx
+++ b/romania-deficit/Model_DSA_Romania.xlsx
@@ -50,10 +50,10 @@
     <t>S1 Nicio schimbare de politică (no-policy change)</t>
   </si>
   <si>
-    <t>S2 Consolidare conform planului (EDP)</t>
+    <t>S2 Consolidare conform planului (PDE)</t>
   </si>
   <si>
-    <t>S3 Derapaj: ajustare amânată + randamente +100bp</t>
+    <t>S3 Derapaj: ajustare amânată + randamente +100 pb</t>
   </si>
   <si>
     <t>S4 Șoc sever 2028 (r-g reversat)</t>

</xml_diff>

<commit_message>
romania-deficit: editia din 17 octombrie 2026 (spatiul fiscal pentru cheltuieli noi, §8.6)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/romania-deficit/Model_DSA_Romania.xlsx
+++ b/romania-deficit/Model_DSA_Romania.xlsx
@@ -25,14 +25,18 @@
     <sheet name="S7 variante" sheetId="16" r:id="rId16"/>
     <sheet name="Dezindustrializare" sheetId="17" r:id="rId17"/>
     <sheet name="Dezindustrializare canale" sheetId="18" r:id="rId18"/>
-    <sheet name="Grafic datorie" sheetId="19" r:id="rId19"/>
+    <sheet name="Spațiu fiscal baze" sheetId="19" r:id="rId19"/>
+    <sheet name="Spațiu fiscal criterii" sheetId="20" r:id="rId20"/>
+    <sheet name="Spațiu fiscal pachete" sheetId="21" r:id="rId21"/>
+    <sheet name="Pensii și salarii" sheetId="22" r:id="rId22"/>
+    <sheet name="Grafic datorie" sheetId="23" r:id="rId23"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="207">
   <si>
     <t>Scenariu</t>
   </si>
@@ -464,6 +468,171 @@
   </si>
   <si>
     <t>Total față de S2</t>
+  </si>
+  <si>
+    <t>baza</t>
+  </si>
+  <si>
+    <t>variatie_deficit_pp</t>
+  </si>
+  <si>
+    <t>variatie_dobanzi_pp</t>
+  </si>
+  <si>
+    <t>spatiu_fata_de_anul_anterior_pp</t>
+  </si>
+  <si>
+    <t>spatiu_fata_de_anul_anterior_mld</t>
+  </si>
+  <si>
+    <t>spatiu_fata_de_2026_pp</t>
+  </si>
+  <si>
+    <t>spatiu_fata_de_2026_mld</t>
+  </si>
+  <si>
+    <t>masuri_noi_cerute_de_program_pp</t>
+  </si>
+  <si>
+    <t>masuri_noi_cerute_de_program_mld</t>
+  </si>
+  <si>
+    <t>B1 Doar măsurile Bolojan (CF, ian. 2026: deficit primar 2,3%)</t>
+  </si>
+  <si>
+    <t>B2 Doar măsurile Bolojan (CF, sept. 2026: deficit 5,5% în 2027)</t>
+  </si>
+  <si>
+    <t>B3 Programul de guvernare (S2: 5,2% în 2027)</t>
+  </si>
+  <si>
+    <t>profil</t>
+  </si>
+  <si>
+    <t>criteriu</t>
+  </si>
+  <si>
+    <t>spatiu_pp_pib</t>
+  </si>
+  <si>
+    <t>spatiu_mld_lei_2027</t>
+  </si>
+  <si>
+    <t>spatiu_mld_lei_2028</t>
+  </si>
+  <si>
+    <t>B4 Program cu taxe înghețate și pensii indexate (S7: 5,5% în 2027)</t>
+  </si>
+  <si>
+    <t>permanent</t>
+  </si>
+  <si>
+    <t>electoral</t>
+  </si>
+  <si>
+    <t>K0 Țintele de deficit din program (5,2/4,2/3,2/2,8%)</t>
+  </si>
+  <si>
+    <t>K1 Deficitul nu crește de la un an la altul (2027–2030)</t>
+  </si>
+  <si>
+    <t>K2 Deficit sub 3% în 2030 (PDE închisă la termen)</t>
+  </si>
+  <si>
+    <t>K3 Datoria scade în fiecare an din 2031 până în 2040</t>
+  </si>
+  <si>
+    <t>varianta</t>
+  </si>
+  <si>
+    <t>cheltuieli_2027_mld</t>
+  </si>
+  <si>
+    <t>cheltuieli_2027_2030_mld</t>
+  </si>
+  <si>
+    <t>deficit_2027</t>
+  </si>
+  <si>
+    <t>deficit_2028</t>
+  </si>
+  <si>
+    <t>deficit_2030</t>
+  </si>
+  <si>
+    <t>inchidere_pde</t>
+  </si>
+  <si>
+    <t>varf_datorie</t>
+  </si>
+  <si>
+    <t>an_varf</t>
+  </si>
+  <si>
+    <t>datorie_2030</t>
+  </si>
+  <si>
+    <t>datorie_2035</t>
+  </si>
+  <si>
+    <t>datorie_2040</t>
+  </si>
+  <si>
+    <t>sub_60_din</t>
+  </si>
+  <si>
+    <t>dobanzi_2035_%pib</t>
+  </si>
+  <si>
+    <t>B3</t>
+  </si>
+  <si>
+    <t>B4</t>
+  </si>
+  <si>
+    <t>B2</t>
+  </si>
+  <si>
+    <t>fără cheltuieli suplimentare</t>
+  </si>
+  <si>
+    <t>Mic (0,25 pp ≈ 5,5 mld. lei/an); 2027–2028, retras din 2029</t>
+  </si>
+  <si>
+    <t>Mic (0,25 pp ≈ 5,5 mld. lei/an); permanent</t>
+  </si>
+  <si>
+    <t>Mediu (0,5 pp ≈ 11 mld. lei/an); 2027–2028, retras din 2029</t>
+  </si>
+  <si>
+    <t>Mediu (0,5 pp ≈ 11 mld. lei/an); permanent</t>
+  </si>
+  <si>
+    <t>Mare (1,0 pp ≈ 22 mld. lei/an), ca în 2023–2024; 2027–2028, retras din 2029</t>
+  </si>
+  <si>
+    <t>Mare (1,0 pp ≈ 22 mld. lei/an), ca în 2023–2024; permanent</t>
+  </si>
+  <si>
+    <t>Mare (1,0 pp ≈ 22 mld. lei/an), ca în 2023–2024; permanent, randamente +50 pb</t>
+  </si>
+  <si>
+    <t>cost_pp_indexare_mld</t>
+  </si>
+  <si>
+    <t>cost_pp_pib</t>
+  </si>
+  <si>
+    <t>Pensii indexate după formulă (7,3%)</t>
+  </si>
+  <si>
+    <t>Pensii +12%</t>
+  </si>
+  <si>
+    <t>Salarii bugetare +10%</t>
+  </si>
+  <si>
+    <t>Pensii +12% și salarii bugetare +10%</t>
   </si>
   <si>
     <t>An</t>
@@ -12700,428 +12869,619 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>144</v>
       </c>
       <c r="B1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1" t="s">
         <v>145</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>146</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>147</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>148</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>149</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>150</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2">
-        <v>2026</v>
+      <c r="K1" t="s">
+        <v>152</v>
+      </c>
+      <c r="L1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" t="s">
+        <v>153</v>
       </c>
       <c r="B2">
-        <v>62.58890458136189</v>
+        <v>2027</v>
       </c>
       <c r="C2">
-        <v>62.58890458136189</v>
+        <v>5.73365081290331</v>
       </c>
       <c r="D2">
-        <v>62.58890458136189</v>
+        <v>-0.2663491870966901</v>
       </c>
       <c r="E2">
-        <v>62.58890458136189</v>
+        <v>0.354261060928406</v>
       </c>
       <c r="F2">
-        <v>62.58890458136189</v>
+        <v>0.2663491870966901</v>
       </c>
       <c r="G2">
-        <v>62.58890458136189</v>
+        <v>5.857598053595286</v>
       </c>
       <c r="H2">
-        <v>62.58890458136189</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3">
+        <v>0.2663491870966901</v>
+      </c>
+      <c r="I2">
+        <v>5.857598053595286</v>
+      </c>
+      <c r="J2">
+        <v>0.5336508129033097</v>
+      </c>
+      <c r="K2">
+        <v>11.73614230640471</v>
+      </c>
+      <c r="L2">
+        <v>64.93452689744312</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" t="s">
+        <v>153</v>
+      </c>
+      <c r="B3">
+        <v>2028</v>
+      </c>
+      <c r="C3">
+        <v>5.972097037934352</v>
+      </c>
+      <c r="D3">
+        <v>0.2384462250310424</v>
+      </c>
+      <c r="E3">
+        <v>0.2384462250310428</v>
+      </c>
+      <c r="F3">
+        <v>-0.2384462250310424</v>
+      </c>
+      <c r="G3">
+        <v>-5.567328207943027</v>
+      </c>
+      <c r="H3">
+        <v>0.02790296206564769</v>
+      </c>
+      <c r="I3">
+        <v>0.6514883922906344</v>
+      </c>
+      <c r="J3">
+        <v>1.74191867731507</v>
+      </c>
+      <c r="K3">
+        <v>40.67094367669891</v>
+      </c>
+      <c r="L3">
+        <v>67.58446344622884</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" t="s">
+        <v>153</v>
+      </c>
+      <c r="B4">
+        <v>2029</v>
+      </c>
+      <c r="C4">
+        <v>6.164868395490132</v>
+      </c>
+      <c r="D4">
+        <v>0.1927713575557792</v>
+      </c>
+      <c r="E4">
+        <v>0.1927713575557788</v>
+      </c>
+      <c r="F4">
+        <v>-0.1927713575557792</v>
+      </c>
+      <c r="G4">
+        <v>-4.76344718433312</v>
+      </c>
+      <c r="H4">
+        <v>-0.1648683954901315</v>
+      </c>
+      <c r="I4">
+        <v>-4.073955302492198</v>
+      </c>
+      <c r="J4">
+        <v>2.834573782584067</v>
+      </c>
+      <c r="K4">
+        <v>70.04330246275093</v>
+      </c>
+      <c r="L4">
+        <v>70.49357005145103</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" t="s">
+        <v>153</v>
+      </c>
+      <c r="B5">
+        <v>2030</v>
+      </c>
+      <c r="C5">
+        <v>6.31596392134774</v>
+      </c>
+      <c r="D5">
+        <v>0.1510955258576088</v>
+      </c>
+      <c r="E5">
+        <v>0.1510955258576092</v>
+      </c>
+      <c r="F5">
+        <v>-0.1510955258576088</v>
+      </c>
+      <c r="G5">
+        <v>-3.938972171416557</v>
+      </c>
+      <c r="H5">
+        <v>-0.3159639213477403</v>
+      </c>
+      <c r="I5">
+        <v>-8.236995015545826</v>
+      </c>
+      <c r="J5">
+        <v>3.223509355352173</v>
+      </c>
+      <c r="K5">
+        <v>84.03500747599226</v>
+      </c>
+      <c r="L5">
+        <v>73.62563007426643</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" t="s">
+        <v>153</v>
+      </c>
+      <c r="B6">
+        <v>2031</v>
+      </c>
+      <c r="C6">
+        <v>6.452482933347304</v>
+      </c>
+      <c r="D6">
+        <v>0.1365190119995638</v>
+      </c>
+      <c r="E6">
+        <v>0.1365190119995638</v>
+      </c>
+      <c r="F6">
+        <v>-0.1365190119995638</v>
+      </c>
+      <c r="G6">
+        <v>-3.736919510935405</v>
+      </c>
+      <c r="H6">
+        <v>-0.4524829333473042</v>
+      </c>
+      <c r="I6">
+        <v>-12.38576427725852</v>
+      </c>
+      <c r="J6">
+        <v>3.477727423253568</v>
+      </c>
+      <c r="K6">
+        <v>95.19544033700514</v>
+      </c>
+      <c r="L6">
+        <v>76.91571689680475</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" t="s">
+        <v>154</v>
+      </c>
+      <c r="B7">
         <v>2027</v>
       </c>
-      <c r="B3">
-        <v>64.93452689744312</v>
-      </c>
-      <c r="C3">
+      <c r="C7">
+        <v>5.5</v>
+      </c>
+      <c r="D7">
+        <v>-0.5</v>
+      </c>
+      <c r="E7">
+        <v>0.354261060928406</v>
+      </c>
+      <c r="F7">
+        <v>0.5</v>
+      </c>
+      <c r="G7">
+        <v>10.996087725</v>
+      </c>
+      <c r="H7">
+        <v>0.5</v>
+      </c>
+      <c r="I7">
+        <v>10.996087725</v>
+      </c>
+      <c r="J7">
+        <v>0.2999999999999998</v>
+      </c>
+      <c r="K7">
+        <v>6.597652634999998</v>
+      </c>
+      <c r="L7">
+        <v>64.70087608453981</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" t="s">
+        <v>154</v>
+      </c>
+      <c r="B8">
+        <v>2028</v>
+      </c>
+      <c r="C8">
+        <v>5.725233093297161</v>
+      </c>
+      <c r="D8">
+        <v>0.2252330932971613</v>
+      </c>
+      <c r="E8">
+        <v>0.2252330932971613</v>
+      </c>
+      <c r="F8">
+        <v>-0.2252330932971613</v>
+      </c>
+      <c r="G8">
+        <v>-5.258823256741866</v>
+      </c>
+      <c r="H8">
+        <v>0.2747669067028387</v>
+      </c>
+      <c r="I8">
+        <v>6.415356544633138</v>
+      </c>
+      <c r="J8">
+        <v>1.508267864411761</v>
+      </c>
+      <c r="K8">
+        <v>35.21558047555758</v>
+      </c>
+      <c r="L8">
+        <v>67.11590266041915</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" t="s">
+        <v>154</v>
+      </c>
+      <c r="B9">
+        <v>2029</v>
+      </c>
+      <c r="C9">
+        <v>5.904422581485974</v>
+      </c>
+      <c r="D9">
+        <v>0.179189488188813</v>
+      </c>
+      <c r="E9">
+        <v>0.179189488188813</v>
+      </c>
+      <c r="F9">
+        <v>-0.179189488188813</v>
+      </c>
+      <c r="G9">
+        <v>-4.427834476022262</v>
+      </c>
+      <c r="H9">
+        <v>0.09557741851402568</v>
+      </c>
+      <c r="I9">
+        <v>2.361751200381141</v>
+      </c>
+      <c r="J9">
+        <v>2.600922969680757</v>
+      </c>
+      <c r="K9">
+        <v>64.26970974154302</v>
+      </c>
+      <c r="L9">
+        <v>69.7871355373662</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>154</v>
+      </c>
+      <c r="B10">
+        <v>2030</v>
+      </c>
+      <c r="C10">
+        <v>6.042068082986238</v>
+      </c>
+      <c r="D10">
+        <v>0.1376455015002636</v>
+      </c>
+      <c r="E10">
+        <v>0.1376455015002636</v>
+      </c>
+      <c r="F10">
+        <v>-0.1376455015002636</v>
+      </c>
+      <c r="G10">
+        <v>-3.588337886597396</v>
+      </c>
+      <c r="H10">
+        <v>-0.04206808298623788</v>
+      </c>
+      <c r="I10">
+        <v>-1.096690370195292</v>
+      </c>
+      <c r="J10">
+        <v>2.989858542448864</v>
+      </c>
+      <c r="K10">
+        <v>77.94386715511791</v>
+      </c>
+      <c r="L10">
+        <v>72.67720645603443</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" t="s">
+        <v>154</v>
+      </c>
+      <c r="B11">
+        <v>2031</v>
+      </c>
+      <c r="C11">
+        <v>6.165341061904744</v>
+      </c>
+      <c r="D11">
+        <v>0.1232729789185063</v>
+      </c>
+      <c r="E11">
+        <v>0.1232729789185059</v>
+      </c>
+      <c r="F11">
+        <v>-0.1232729789185063</v>
+      </c>
+      <c r="G11">
+        <v>-3.374337342063147</v>
+      </c>
+      <c r="H11">
+        <v>-0.1653410619047442</v>
+      </c>
+      <c r="I11">
+        <v>-4.525862230768204</v>
+      </c>
+      <c r="J11">
+        <v>3.244076610350258</v>
+      </c>
+      <c r="K11">
+        <v>88.79974300008708</v>
+      </c>
+      <c r="L11">
+        <v>75.72088845968473</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>155</v>
+      </c>
+      <c r="B12">
+        <v>2027</v>
+      </c>
+      <c r="C12">
+        <v>5.2</v>
+      </c>
+      <c r="D12">
+        <v>-0.7999999999999998</v>
+      </c>
+      <c r="E12">
+        <v>0.354261060928406</v>
+      </c>
+      <c r="F12">
+        <v>0.7999999999999998</v>
+      </c>
+      <c r="G12">
+        <v>17.59374036</v>
+      </c>
+      <c r="H12">
+        <v>0.7999999999999998</v>
+      </c>
+      <c r="I12">
+        <v>17.59374036</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
         <v>64.40087608453982</v>
       </c>
-      <c r="D3">
-        <v>65.11927783670889</v>
-      </c>
-      <c r="E3">
-        <v>64.40087608453982</v>
-      </c>
-      <c r="F3">
-        <v>64.23452689744312</v>
-      </c>
-      <c r="G3">
-        <v>63.3477288453457</v>
-      </c>
-      <c r="H3">
-        <v>64.70087608453981</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4">
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" t="s">
+        <v>155</v>
+      </c>
+      <c r="B13">
         <v>2028</v>
       </c>
-      <c r="B4">
-        <v>67.58446344622884</v>
-      </c>
-      <c r="C4">
+      <c r="C13">
+        <v>4.2</v>
+      </c>
+      <c r="D13">
+        <v>-1</v>
+      </c>
+      <c r="E13">
+        <v>0.208267864411761</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13">
+        <v>23.34835960275</v>
+      </c>
+      <c r="H13">
+        <v>1.8</v>
+      </c>
+      <c r="I13">
+        <v>42.02704728495001</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="L13">
         <v>65.30601807575621</v>
       </c>
-      <c r="D4">
-        <v>67.61679648032644</v>
-      </c>
-      <c r="E4">
-        <v>71.6510009632115</v>
-      </c>
-      <c r="F4">
-        <v>65.0806910989761</v>
-      </c>
-      <c r="G4">
-        <v>63.46791745915831</v>
-      </c>
-      <c r="H4">
-        <v>65.89066956712199</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5">
+    </row>
+    <row r="14" spans="1:12">
+      <c r="A14" t="s">
+        <v>155</v>
+      </c>
+      <c r="B14">
         <v>2029</v>
       </c>
-      <c r="B5">
-        <v>70.49357005145103</v>
-      </c>
-      <c r="C5">
+      <c r="C14">
+        <v>3.2</v>
+      </c>
+      <c r="D14">
+        <v>-1</v>
+      </c>
+      <c r="E14">
+        <v>0.0926551052689959</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14">
+        <v>24.71034724624376</v>
+      </c>
+      <c r="H14">
+        <v>2.8</v>
+      </c>
+      <c r="I14">
+        <v>69.18897228948251</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14">
         <v>65.36001635459498</v>
       </c>
-      <c r="D5">
-        <v>69.89307888062643</v>
-      </c>
-      <c r="E5">
-        <v>74.05769779985735</v>
-      </c>
-      <c r="F5">
-        <v>65.16723239559157</v>
-      </c>
-      <c r="G5">
-        <v>62.95181813709121</v>
-      </c>
-      <c r="H5">
-        <v>66.21650329616409</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6">
+    </row>
+    <row r="15" spans="1:12">
+      <c r="A15" t="s">
+        <v>155</v>
+      </c>
+      <c r="B15">
         <v>2030</v>
       </c>
-      <c r="B6">
-        <v>73.62563007426643</v>
-      </c>
-      <c r="C6">
+      <c r="C15">
+        <v>2.8</v>
+      </c>
+      <c r="D15">
+        <v>-0.4000000000000004</v>
+      </c>
+      <c r="E15">
+        <v>-0.0110644272318936</v>
+      </c>
+      <c r="F15">
+        <v>0.4000000000000004</v>
+      </c>
+      <c r="G15">
+        <v>10.42776653791487</v>
+      </c>
+      <c r="H15">
+        <v>3.2</v>
+      </c>
+      <c r="I15">
+        <v>83.42213230331892</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15">
         <v>65.20797390976422</v>
       </c>
-      <c r="D6">
-        <v>71.6678292693645</v>
-      </c>
-      <c r="E6">
-        <v>74.64756096677065</v>
-      </c>
-      <c r="F6">
-        <v>64.53642381027402</v>
-      </c>
-      <c r="G6">
-        <v>61.56590024996358</v>
-      </c>
-      <c r="H6">
-        <v>66.32577686766911</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="A7">
+    </row>
+    <row r="16" spans="1:12">
+      <c r="A16" t="s">
+        <v>155</v>
+      </c>
+      <c r="B16">
         <v>2031</v>
       </c>
-      <c r="B7">
-        <v>76.91571689680475</v>
-      </c>
-      <c r="C7">
+      <c r="C16">
+        <v>2.5</v>
+      </c>
+      <c r="D16">
+        <v>-0.2999999999999998</v>
+      </c>
+      <c r="E16">
+        <v>-0.04578193209860526</v>
+      </c>
+      <c r="F16">
+        <v>0.2999999999999998</v>
+      </c>
+      <c r="G16">
+        <v>8.211866148607951</v>
+      </c>
+      <c r="H16">
+        <v>3.5</v>
+      </c>
+      <c r="I16">
+        <v>95.80510506709282</v>
+      </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16">
         <v>64.9071361732591</v>
-      </c>
-      <c r="D7">
-        <v>72.91047367921412</v>
-      </c>
-      <c r="E7">
-        <v>74.99032613545374</v>
-      </c>
-      <c r="F7">
-        <v>64.00428277085403</v>
-      </c>
-      <c r="G7">
-        <v>60.10105472545386</v>
-      </c>
-      <c r="H7">
-        <v>66.27692683268637</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8">
-        <v>2032</v>
-      </c>
-      <c r="B8">
-        <v>80.19217073544627</v>
-      </c>
-      <c r="C8">
-        <v>64.41922013381722</v>
-      </c>
-      <c r="D8">
-        <v>73.57912643541387</v>
-      </c>
-      <c r="E8">
-        <v>75.0456458856188</v>
-      </c>
-      <c r="F8">
-        <v>63.41682447393597</v>
-      </c>
-      <c r="G8">
-        <v>58.56496087171271</v>
-      </c>
-      <c r="H8">
-        <v>66.03017502301574</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="A9">
-        <v>2033</v>
-      </c>
-      <c r="B9">
-        <v>83.46194582525446</v>
-      </c>
-      <c r="C9">
-        <v>63.75226124997421</v>
-      </c>
-      <c r="D9">
-        <v>73.88919028036351</v>
-      </c>
-      <c r="E9">
-        <v>74.83962172719177</v>
-      </c>
-      <c r="F9">
-        <v>62.78373296494627</v>
-      </c>
-      <c r="G9">
-        <v>56.9756007575451</v>
-      </c>
-      <c r="H9">
-        <v>65.59402179107478</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10">
-        <v>2034</v>
-      </c>
-      <c r="B10">
-        <v>86.73106913700117</v>
-      </c>
-      <c r="C10">
-        <v>63.0139498381896</v>
-      </c>
-      <c r="D10">
-        <v>73.94867584698677</v>
-      </c>
-      <c r="E10">
-        <v>74.49526406304325</v>
-      </c>
-      <c r="F10">
-        <v>62.11274998717341</v>
-      </c>
-      <c r="G10">
-        <v>55.34721584948421</v>
-      </c>
-      <c r="H10">
-        <v>65.07660237890576</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11">
-        <v>2035</v>
-      </c>
-      <c r="B11">
-        <v>90.00473769204891</v>
-      </c>
-      <c r="C11">
-        <v>62.30735065942545</v>
-      </c>
-      <c r="D11">
-        <v>73.8623589199684</v>
-      </c>
-      <c r="E11">
-        <v>74.12875101713996</v>
-      </c>
-      <c r="F11">
-        <v>61.41004603265997</v>
-      </c>
-      <c r="G11">
-        <v>53.69103706293036</v>
-      </c>
-      <c r="H11">
-        <v>64.58140736244037</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12">
-        <v>2036</v>
-      </c>
-      <c r="B12">
-        <v>93.28741693369645</v>
-      </c>
-      <c r="C12">
-        <v>61.63110159776822</v>
-      </c>
-      <c r="D12">
-        <v>73.73198829228667</v>
-      </c>
-      <c r="E12">
-        <v>73.74969255356471</v>
-      </c>
-      <c r="F12">
-        <v>60.6805260430722</v>
-      </c>
-      <c r="G12">
-        <v>52.01588866560481</v>
-      </c>
-      <c r="H12">
-        <v>64.10748215096793</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8">
-      <c r="A13">
-        <v>2037</v>
-      </c>
-      <c r="B13">
-        <v>96.58293494872801</v>
-      </c>
-      <c r="C13">
-        <v>60.98389904342599</v>
-      </c>
-      <c r="D13">
-        <v>73.55642246441616</v>
-      </c>
-      <c r="E13">
-        <v>73.36562480500363</v>
-      </c>
-      <c r="F13">
-        <v>59.92807915176644</v>
-      </c>
-      <c r="G13">
-        <v>50.32868136290389</v>
-      </c>
-      <c r="H13">
-        <v>63.65391315572158</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
-      <c r="A14">
-        <v>2038</v>
-      </c>
-      <c r="B14">
-        <v>99.89456963935189</v>
-      </c>
-      <c r="C14">
-        <v>60.36449537975121</v>
-      </c>
-      <c r="D14">
-        <v>73.33513102609251</v>
-      </c>
-      <c r="E14">
-        <v>72.98240193531805</v>
-      </c>
-      <c r="F14">
-        <v>59.15578138347605</v>
-      </c>
-      <c r="G14">
-        <v>48.63481092680315</v>
-      </c>
-      <c r="H14">
-        <v>63.21982602874725</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8">
-      <c r="A15">
-        <v>2039</v>
-      </c>
-      <c r="B15">
-        <v>103.2251274661083</v>
-      </c>
-      <c r="C15">
-        <v>59.7716965782019</v>
-      </c>
-      <c r="D15">
-        <v>73.16805726026966</v>
-      </c>
-      <c r="E15">
-        <v>72.60452330653708</v>
-      </c>
-      <c r="F15">
-        <v>58.36605933674945</v>
-      </c>
-      <c r="G15">
-        <v>46.93847799930541</v>
-      </c>
-      <c r="H15">
-        <v>62.80438397741724</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
-      <c r="A16">
-        <v>2040</v>
-      </c>
-      <c r="B16">
-        <v>106.5770133547019</v>
-      </c>
-      <c r="C16">
-        <v>59.20435989660484</v>
-      </c>
-      <c r="D16">
-        <v>73.05212746939111</v>
-      </c>
-      <c r="E16">
-        <v>72.23540329299968</v>
-      </c>
-      <c r="F16">
-        <v>57.56082183010944</v>
-      </c>
-      <c r="G16">
-        <v>45.24294311860554</v>
-      </c>
-      <c r="H16">
-        <v>62.4067861513396</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -13374,6 +13734,2132 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D1" t="s">
+        <v>158</v>
+      </c>
+      <c r="E1" t="s">
+        <v>159</v>
+      </c>
+      <c r="F1" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C2" t="s">
+        <v>164</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>155</v>
+      </c>
+      <c r="B3" t="s">
+        <v>162</v>
+      </c>
+      <c r="C3" t="s">
+        <v>165</v>
+      </c>
+      <c r="D3">
+        <v>1.0869140625</v>
+      </c>
+      <c r="E3">
+        <v>23.90360476157227</v>
+      </c>
+      <c r="F3">
+        <v>25.3776603885359</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B4" t="s">
+        <v>162</v>
+      </c>
+      <c r="C4" t="s">
+        <v>166</v>
+      </c>
+      <c r="D4">
+        <v>0.17449951171875</v>
+      </c>
+      <c r="E4">
+        <v>3.837623877658082</v>
+      </c>
+      <c r="F4">
+        <v>4.074277350113664</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
+        <v>155</v>
+      </c>
+      <c r="B5" t="s">
+        <v>162</v>
+      </c>
+      <c r="C5" t="s">
+        <v>167</v>
+      </c>
+      <c r="D5">
+        <v>0.28692626953125</v>
+      </c>
+      <c r="E5">
+        <v>6.31013286074524</v>
+      </c>
+      <c r="F5">
+        <v>6.699257720491197</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>155</v>
+      </c>
+      <c r="B6" t="s">
+        <v>163</v>
+      </c>
+      <c r="C6" t="s">
+        <v>164</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
+        <v>155</v>
+      </c>
+      <c r="B7" t="s">
+        <v>163</v>
+      </c>
+      <c r="C7" t="s">
+        <v>165</v>
+      </c>
+      <c r="D7">
+        <v>1.0869140625</v>
+      </c>
+      <c r="E7">
+        <v>23.90360476157227</v>
+      </c>
+      <c r="F7">
+        <v>25.3776603885359</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" t="s">
+        <v>155</v>
+      </c>
+      <c r="B8" t="s">
+        <v>163</v>
+      </c>
+      <c r="C8" t="s">
+        <v>166</v>
+      </c>
+      <c r="D8">
+        <v>0.71173095703125</v>
+      </c>
+      <c r="E8">
+        <v>15.65251208022766</v>
+      </c>
+      <c r="F8">
+        <v>16.61775032517504</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" t="s">
+        <v>155</v>
+      </c>
+      <c r="B9" t="s">
+        <v>163</v>
+      </c>
+      <c r="C9" t="s">
+        <v>167</v>
+      </c>
+      <c r="D9">
+        <v>6</v>
+      </c>
+      <c r="E9">
+        <v>131.9530527</v>
+      </c>
+      <c r="F9">
+        <v>140.0901576165</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" t="s">
+        <v>161</v>
+      </c>
+      <c r="B10" t="s">
+        <v>162</v>
+      </c>
+      <c r="C10" t="s">
+        <v>165</v>
+      </c>
+      <c r="D10">
+        <v>0.6793212890625</v>
+      </c>
+      <c r="E10">
+        <v>14.93975297598267</v>
+      </c>
+      <c r="F10">
+        <v>15.86103774283493</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" t="s">
+        <v>161</v>
+      </c>
+      <c r="B11" t="s">
+        <v>162</v>
+      </c>
+      <c r="C11" t="s">
+        <v>166</v>
+      </c>
+      <c r="D11">
+        <v>-0.08734130859375</v>
+      </c>
+      <c r="E11">
+        <v>-1.920825382626343</v>
+      </c>
+      <c r="F11">
+        <v>-2.039276281221635</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" t="s">
+        <v>161</v>
+      </c>
+      <c r="B12" t="s">
+        <v>162</v>
+      </c>
+      <c r="C12" t="s">
+        <v>167</v>
+      </c>
+      <c r="D12">
+        <v>0.0465087890625</v>
+      </c>
+      <c r="E12">
+        <v>1.022829449029541</v>
+      </c>
+      <c r="F12">
+        <v>1.085903931719696</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" t="s">
+        <v>161</v>
+      </c>
+      <c r="B13" t="s">
+        <v>163</v>
+      </c>
+      <c r="C13" t="s">
+        <v>165</v>
+      </c>
+      <c r="D13">
+        <v>0.6793212890625</v>
+      </c>
+      <c r="E13">
+        <v>14.93975297598267</v>
+      </c>
+      <c r="F13">
+        <v>15.86103774283493</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" t="s">
+        <v>161</v>
+      </c>
+      <c r="B14" t="s">
+        <v>163</v>
+      </c>
+      <c r="C14" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" t="s">
+        <v>161</v>
+      </c>
+      <c r="B15" t="s">
+        <v>163</v>
+      </c>
+      <c r="C15" t="s">
+        <v>167</v>
+      </c>
+      <c r="D15">
+        <v>6</v>
+      </c>
+      <c r="E15">
+        <v>131.9530527</v>
+      </c>
+      <c r="F15">
+        <v>140.0901576165</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" t="s">
+        <v>154</v>
+      </c>
+      <c r="B16" t="s">
+        <v>162</v>
+      </c>
+      <c r="C16" t="s">
+        <v>166</v>
+      </c>
+      <c r="D16">
+        <v>-2.6583251953125</v>
+      </c>
+      <c r="E16">
+        <v>-58.46235409846803</v>
+      </c>
+      <c r="F16">
+        <v>-62.0675326012069</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" t="s">
+        <v>154</v>
+      </c>
+      <c r="B17" t="s">
+        <v>162</v>
+      </c>
+      <c r="C17" t="s">
+        <v>167</v>
+      </c>
+      <c r="D17">
+        <v>-2.90460205078125</v>
+      </c>
+      <c r="E17">
+        <v>-63.87851791321107</v>
+      </c>
+      <c r="F17">
+        <v>-67.81769318452575</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" t="s">
+        <v>153</v>
+      </c>
+      <c r="B18" t="s">
+        <v>162</v>
+      </c>
+      <c r="C18" t="s">
+        <v>166</v>
+      </c>
+      <c r="D18">
+        <v>-2.89764404296875</v>
+      </c>
+      <c r="E18">
+        <v>-63.7254961846161</v>
+      </c>
+      <c r="F18">
+        <v>-67.65523511600077</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" t="s">
+        <v>153</v>
+      </c>
+      <c r="B19" t="s">
+        <v>162</v>
+      </c>
+      <c r="C19" t="s">
+        <v>167</v>
+      </c>
+      <c r="D19">
+        <v>-3.139801025390625</v>
+      </c>
+      <c r="E19">
+        <v>-69.05105502848053</v>
+      </c>
+      <c r="F19">
+        <v>-73.3092034219035</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:O13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:15">
+      <c r="A1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C1" t="s">
+        <v>169</v>
+      </c>
+      <c r="D1" t="s">
+        <v>170</v>
+      </c>
+      <c r="E1" t="s">
+        <v>171</v>
+      </c>
+      <c r="F1" t="s">
+        <v>172</v>
+      </c>
+      <c r="G1" t="s">
+        <v>173</v>
+      </c>
+      <c r="H1" t="s">
+        <v>174</v>
+      </c>
+      <c r="I1" t="s">
+        <v>175</v>
+      </c>
+      <c r="J1" t="s">
+        <v>176</v>
+      </c>
+      <c r="K1" t="s">
+        <v>177</v>
+      </c>
+      <c r="L1" t="s">
+        <v>178</v>
+      </c>
+      <c r="M1" t="s">
+        <v>179</v>
+      </c>
+      <c r="N1" t="s">
+        <v>180</v>
+      </c>
+      <c r="O1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
+      <c r="A2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B2" t="s">
+        <v>185</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>5.2</v>
+      </c>
+      <c r="F2">
+        <v>4.2</v>
+      </c>
+      <c r="G2">
+        <v>2.8</v>
+      </c>
+      <c r="H2">
+        <v>2030</v>
+      </c>
+      <c r="I2">
+        <v>65.36001635459498</v>
+      </c>
+      <c r="J2">
+        <v>2029</v>
+      </c>
+      <c r="K2">
+        <v>65.20797390976422</v>
+      </c>
+      <c r="L2">
+        <v>62.30735065942545</v>
+      </c>
+      <c r="M2">
+        <v>59.20435989660484</v>
+      </c>
+      <c r="N2">
+        <v>2039</v>
+      </c>
+      <c r="O2">
+        <v>3.414012359499693</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
+      <c r="A3" t="s">
+        <v>182</v>
+      </c>
+      <c r="B3" t="s">
+        <v>186</v>
+      </c>
+      <c r="C3">
+        <v>5.507723517187501</v>
+      </c>
+      <c r="D3">
+        <v>11.35164765740332</v>
+      </c>
+      <c r="E3">
+        <v>5.383965464300697</v>
+      </c>
+      <c r="F3">
+        <v>4.416667547503584</v>
+      </c>
+      <c r="G3">
+        <v>2.870097416965697</v>
+      </c>
+      <c r="H3">
+        <v>2030</v>
+      </c>
+      <c r="I3">
+        <v>65.88832647211392</v>
+      </c>
+      <c r="J3">
+        <v>2029</v>
+      </c>
+      <c r="K3">
+        <v>65.78251985458083</v>
+      </c>
+      <c r="L3">
+        <v>62.85640556686793</v>
+      </c>
+      <c r="M3">
+        <v>59.78289218922298</v>
+      </c>
+      <c r="N3">
+        <v>2040</v>
+      </c>
+      <c r="O3">
+        <v>3.443429185368529</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15">
+      <c r="A4" t="s">
+        <v>182</v>
+      </c>
+      <c r="B4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C4">
+        <v>5.507723517187501</v>
+      </c>
+      <c r="D4">
+        <v>24.05008315224857</v>
+      </c>
+      <c r="E4">
+        <v>5.383965464300697</v>
+      </c>
+      <c r="F4">
+        <v>4.416667547503584</v>
+      </c>
+      <c r="G4">
+        <v>3.0864450635383</v>
+      </c>
+      <c r="H4">
+        <v>2031</v>
+      </c>
+      <c r="I4">
+        <v>66.10525739409731</v>
+      </c>
+      <c r="J4">
+        <v>2030</v>
+      </c>
+      <c r="K4">
+        <v>66.10525739409731</v>
+      </c>
+      <c r="L4">
+        <v>64.54029242721926</v>
+      </c>
+      <c r="M4">
+        <v>62.83328558740713</v>
+      </c>
+      <c r="O4">
+        <v>3.520252831810457</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15">
+      <c r="A5" t="s">
+        <v>182</v>
+      </c>
+      <c r="B5" t="s">
+        <v>188</v>
+      </c>
+      <c r="C5">
+        <v>11.03480634375</v>
+      </c>
+      <c r="D5">
+        <v>22.73629890410157</v>
+      </c>
+      <c r="E5">
+        <v>5.567952102410866</v>
+      </c>
+      <c r="F5">
+        <v>4.633364822476611</v>
+      </c>
+      <c r="G5">
+        <v>2.940357408875622</v>
+      </c>
+      <c r="H5">
+        <v>2030</v>
+      </c>
+      <c r="I5">
+        <v>66.41949032249603</v>
+      </c>
+      <c r="J5">
+        <v>2029</v>
+      </c>
+      <c r="K5">
+        <v>66.35995321585797</v>
+      </c>
+      <c r="L5">
+        <v>63.40719276417168</v>
+      </c>
+      <c r="M5">
+        <v>60.36324977401379</v>
+      </c>
+      <c r="O5">
+        <v>3.472938822481763</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15">
+      <c r="A6" t="s">
+        <v>182</v>
+      </c>
+      <c r="B6" t="s">
+        <v>189</v>
+      </c>
+      <c r="C6">
+        <v>11.03480634375</v>
+      </c>
+      <c r="D6">
+        <v>48.14006251133094</v>
+      </c>
+      <c r="E6">
+        <v>5.567952102410866</v>
+      </c>
+      <c r="F6">
+        <v>4.633364822476611</v>
+      </c>
+      <c r="G6">
+        <v>3.372988809557949</v>
+      </c>
+      <c r="H6">
+        <v>2032</v>
+      </c>
+      <c r="I6">
+        <v>67.26915461956719</v>
+      </c>
+      <c r="J6">
+        <v>2032</v>
+      </c>
+      <c r="K6">
+        <v>67.00429353116765</v>
+      </c>
+      <c r="L6">
+        <v>66.77509653299165</v>
+      </c>
+      <c r="M6">
+        <v>66.46417360045764</v>
+      </c>
+      <c r="O6">
+        <v>3.626593082979914</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15">
+      <c r="A7" t="s">
+        <v>182</v>
+      </c>
+      <c r="B7" t="s">
+        <v>190</v>
+      </c>
+      <c r="C7">
+        <v>22.147049925</v>
+      </c>
+      <c r="D7">
+        <v>45.60446697056251</v>
+      </c>
+      <c r="E7">
+        <v>5.935988455853823</v>
+      </c>
+      <c r="F7">
+        <v>5.066848306024109</v>
+      </c>
+      <c r="G7">
+        <v>3.08136951321595</v>
+      </c>
+      <c r="H7">
+        <v>2031</v>
+      </c>
+      <c r="I7">
+        <v>67.52356025751943</v>
+      </c>
+      <c r="J7">
+        <v>2030</v>
+      </c>
+      <c r="K7">
+        <v>67.52356025751943</v>
+      </c>
+      <c r="L7">
+        <v>64.51401727002384</v>
+      </c>
+      <c r="M7">
+        <v>61.52949692018595</v>
+      </c>
+      <c r="O7">
+        <v>3.532239382980668</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15">
+      <c r="A8" t="s">
+        <v>182</v>
+      </c>
+      <c r="B8" t="s">
+        <v>191</v>
+      </c>
+      <c r="C8">
+        <v>22.147049925</v>
+      </c>
+      <c r="D8">
+        <v>96.43898658038218</v>
+      </c>
+      <c r="E8">
+        <v>5.935988455853823</v>
+      </c>
+      <c r="F8">
+        <v>5.066848306024109</v>
+      </c>
+      <c r="G8">
+        <v>3.946373191114821</v>
+      </c>
+      <c r="I8">
+        <v>73.73185333811564</v>
+      </c>
+      <c r="J8">
+        <v>2040</v>
+      </c>
+      <c r="K8">
+        <v>68.80763871918859</v>
+      </c>
+      <c r="L8">
+        <v>71.25030765010257</v>
+      </c>
+      <c r="M8">
+        <v>73.73185333811564</v>
+      </c>
+      <c r="O8">
+        <v>3.839573773324008</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15">
+      <c r="A9" t="s">
+        <v>182</v>
+      </c>
+      <c r="B9" t="s">
+        <v>192</v>
+      </c>
+      <c r="C9">
+        <v>22.147049925</v>
+      </c>
+      <c r="D9">
+        <v>96.43898658038218</v>
+      </c>
+      <c r="E9">
+        <v>5.994775339797911</v>
+      </c>
+      <c r="F9">
+        <v>5.181082923045763</v>
+      </c>
+      <c r="G9">
+        <v>4.15747535369572</v>
+      </c>
+      <c r="I9">
+        <v>77.44182723879656</v>
+      </c>
+      <c r="J9">
+        <v>2040</v>
+      </c>
+      <c r="K9">
+        <v>69.33226628649075</v>
+      </c>
+      <c r="L9">
+        <v>73.16331939091617</v>
+      </c>
+      <c r="M9">
+        <v>77.44182723879656</v>
+      </c>
+      <c r="O9">
+        <v>4.2261978268449</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15">
+      <c r="A10" t="s">
+        <v>183</v>
+      </c>
+      <c r="B10" t="s">
+        <v>185</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>5.5</v>
+      </c>
+      <c r="F10">
+        <v>4.5</v>
+      </c>
+      <c r="G10">
+        <v>3.1</v>
+      </c>
+      <c r="H10">
+        <v>2031</v>
+      </c>
+      <c r="I10">
+        <v>66.32577686766911</v>
+      </c>
+      <c r="J10">
+        <v>2030</v>
+      </c>
+      <c r="K10">
+        <v>66.32577686766911</v>
+      </c>
+      <c r="L10">
+        <v>64.58140736244037</v>
+      </c>
+      <c r="M10">
+        <v>62.4067861513396</v>
+      </c>
+      <c r="O10">
+        <v>3.525764142802295</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15">
+      <c r="A11" t="s">
+        <v>183</v>
+      </c>
+      <c r="B11" t="s">
+        <v>189</v>
+      </c>
+      <c r="C11">
+        <v>11.03480634375</v>
+      </c>
+      <c r="D11">
+        <v>48.14006251133094</v>
+      </c>
+      <c r="E11">
+        <v>5.867952102410865</v>
+      </c>
+      <c r="F11">
+        <v>4.93338482078178</v>
+      </c>
+      <c r="G11">
+        <v>3.673106963828753</v>
+      </c>
+      <c r="I11">
+        <v>69.66894937813868</v>
+      </c>
+      <c r="J11">
+        <v>2040</v>
+      </c>
+      <c r="K11">
+        <v>68.12419497102508</v>
+      </c>
+      <c r="L11">
+        <v>69.05138304602799</v>
+      </c>
+      <c r="M11">
+        <v>69.66894937813868</v>
+      </c>
+      <c r="O11">
+        <v>3.738464333265201</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15">
+      <c r="A12" t="s">
+        <v>184</v>
+      </c>
+      <c r="B12" t="s">
+        <v>185</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>5.5</v>
+      </c>
+      <c r="F12">
+        <v>5.725233093297161</v>
+      </c>
+      <c r="G12">
+        <v>6.042068082986238</v>
+      </c>
+      <c r="I12">
+        <v>103.0624503556087</v>
+      </c>
+      <c r="J12">
+        <v>2040</v>
+      </c>
+      <c r="K12">
+        <v>72.67720645603443</v>
+      </c>
+      <c r="L12">
+        <v>87.80113072598846</v>
+      </c>
+      <c r="M12">
+        <v>103.0624503556087</v>
+      </c>
+      <c r="O12">
+        <v>4.593429737619568</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15">
+      <c r="A13" t="s">
+        <v>184</v>
+      </c>
+      <c r="B13" t="s">
+        <v>189</v>
+      </c>
+      <c r="C13">
+        <v>11.03480634375</v>
+      </c>
+      <c r="D13">
+        <v>48.14006251133094</v>
+      </c>
+      <c r="E13">
+        <v>5.867952102410865</v>
+      </c>
+      <c r="F13">
+        <v>6.158617914078941</v>
+      </c>
+      <c r="G13">
+        <v>6.615499728898881</v>
+      </c>
+      <c r="I13">
+        <v>110.3310699550903</v>
+      </c>
+      <c r="J13">
+        <v>2040</v>
+      </c>
+      <c r="K13">
+        <v>74.48139108385648</v>
+      </c>
+      <c r="L13">
+        <v>92.27723381707061</v>
+      </c>
+      <c r="M13">
+        <v>110.3310699550903</v>
+      </c>
+      <c r="O13">
+        <v>4.806458217433596</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Q15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:17">
+      <c r="A1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B1" t="s">
+        <v>193</v>
+      </c>
+      <c r="C1" t="s">
+        <v>194</v>
+      </c>
+      <c r="D1" t="s">
+        <v>168</v>
+      </c>
+      <c r="E1" t="s">
+        <v>169</v>
+      </c>
+      <c r="F1" t="s">
+        <v>170</v>
+      </c>
+      <c r="G1" t="s">
+        <v>171</v>
+      </c>
+      <c r="H1" t="s">
+        <v>172</v>
+      </c>
+      <c r="I1" t="s">
+        <v>173</v>
+      </c>
+      <c r="J1" t="s">
+        <v>174</v>
+      </c>
+      <c r="K1" t="s">
+        <v>175</v>
+      </c>
+      <c r="L1" t="s">
+        <v>176</v>
+      </c>
+      <c r="M1" t="s">
+        <v>177</v>
+      </c>
+      <c r="N1" t="s">
+        <v>178</v>
+      </c>
+      <c r="O1" t="s">
+        <v>179</v>
+      </c>
+      <c r="P1" t="s">
+        <v>180</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17">
+      <c r="A2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>0.03637657410558716</v>
+      </c>
+      <c r="D2" t="s">
+        <v>195</v>
+      </c>
+      <c r="E2">
+        <v>0.8002049384456651</v>
+      </c>
+      <c r="F2">
+        <v>3.496951334826595</v>
+      </c>
+      <c r="G2">
+        <v>5.526766812768926</v>
+      </c>
+      <c r="H2">
+        <v>5.756759188554835</v>
+      </c>
+      <c r="I2">
+        <v>6.083773685831616</v>
+      </c>
+      <c r="K2">
+        <v>103.5909997539785</v>
+      </c>
+      <c r="L2">
+        <v>2040</v>
+      </c>
+      <c r="M2">
+        <v>72.80822938154994</v>
+      </c>
+      <c r="N2">
+        <v>88.12652928778991</v>
+      </c>
+      <c r="O2">
+        <v>103.5909997539785</v>
+      </c>
+      <c r="Q2">
+        <v>4.60891472713349</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17">
+      <c r="A3" t="s">
+        <v>155</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>0.03637657410558716</v>
+      </c>
+      <c r="D3" t="s">
+        <v>195</v>
+      </c>
+      <c r="E3">
+        <v>0.8002049384456651</v>
+      </c>
+      <c r="F3">
+        <v>3.496951334826595</v>
+      </c>
+      <c r="G3">
+        <v>5.226766812768927</v>
+      </c>
+      <c r="H3">
+        <v>4.231524641906558</v>
+      </c>
+      <c r="I3">
+        <v>2.841673433563164</v>
+      </c>
+      <c r="J3">
+        <v>2030</v>
+      </c>
+      <c r="K3">
+        <v>65.44735184120117</v>
+      </c>
+      <c r="L3">
+        <v>2029</v>
+      </c>
+      <c r="M3">
+        <v>65.3384254919191</v>
+      </c>
+      <c r="N3">
+        <v>62.63214212181885</v>
+      </c>
+      <c r="O3">
+        <v>59.73226960191728</v>
+      </c>
+      <c r="P3">
+        <v>2040</v>
+      </c>
+      <c r="Q3">
+        <v>3.429464822325792</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17">
+      <c r="A4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B4">
+        <v>1.55</v>
+      </c>
+      <c r="C4">
+        <v>0.0563836898636601</v>
+      </c>
+      <c r="D4" t="s">
+        <v>195</v>
+      </c>
+      <c r="E4">
+        <v>1.24049236461571</v>
+      </c>
+      <c r="F4">
+        <v>5.420636049271903</v>
+      </c>
+      <c r="G4">
+        <v>5.541488751762014</v>
+      </c>
+      <c r="H4">
+        <v>5.774098809828859</v>
+      </c>
+      <c r="I4">
+        <v>6.106712659549254</v>
+      </c>
+      <c r="K4">
+        <v>103.8817196637287</v>
+      </c>
+      <c r="L4">
+        <v>2040</v>
+      </c>
+      <c r="M4">
+        <v>72.88030783568399</v>
+      </c>
+      <c r="N4">
+        <v>88.30551533350587</v>
+      </c>
+      <c r="O4">
+        <v>103.8817196637287</v>
+      </c>
+      <c r="Q4">
+        <v>4.617432373430777</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17">
+      <c r="A5" t="s">
+        <v>155</v>
+      </c>
+      <c r="B5">
+        <v>1.55</v>
+      </c>
+      <c r="C5">
+        <v>0.0563836898636601</v>
+      </c>
+      <c r="D5" t="s">
+        <v>195</v>
+      </c>
+      <c r="E5">
+        <v>1.24049236461571</v>
+      </c>
+      <c r="F5">
+        <v>5.420636049271903</v>
+      </c>
+      <c r="G5">
+        <v>5.241488751762014</v>
+      </c>
+      <c r="H5">
+        <v>4.248863463731324</v>
+      </c>
+      <c r="I5">
+        <v>2.864594710938828</v>
+      </c>
+      <c r="J5">
+        <v>2030</v>
+      </c>
+      <c r="K5">
+        <v>65.4953951276557</v>
+      </c>
+      <c r="L5">
+        <v>2029</v>
+      </c>
+      <c r="M5">
+        <v>65.41018964971833</v>
+      </c>
+      <c r="N5">
+        <v>62.81079420177629</v>
+      </c>
+      <c r="O5">
+        <v>60.02263761612242</v>
+      </c>
+      <c r="Q5">
+        <v>3.437964575672062</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17">
+      <c r="A6" t="s">
+        <v>154</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>0.2500889469759118</v>
+      </c>
+      <c r="D6" t="s">
+        <v>196</v>
+      </c>
+      <c r="E6">
+        <v>5.509686543720898</v>
+      </c>
+      <c r="F6">
+        <v>24.05864699147237</v>
+      </c>
+      <c r="G6">
+        <v>5.684030920762236</v>
+      </c>
+      <c r="H6">
+        <v>5.941987730607419</v>
+      </c>
+      <c r="I6">
+        <v>6.328836395023378</v>
+      </c>
+      <c r="K6">
+        <v>106.6970684643154</v>
+      </c>
+      <c r="L6">
+        <v>2040</v>
+      </c>
+      <c r="M6">
+        <v>73.57874020554186</v>
+      </c>
+      <c r="N6">
+        <v>90.03904398290364</v>
+      </c>
+      <c r="O6">
+        <v>106.6970684643154</v>
+      </c>
+      <c r="Q6">
+        <v>4.699931802878765</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17">
+      <c r="A7" t="s">
+        <v>155</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>0.2500889469759118</v>
+      </c>
+      <c r="D7" t="s">
+        <v>196</v>
+      </c>
+      <c r="E7">
+        <v>5.509686543720898</v>
+      </c>
+      <c r="F7">
+        <v>24.05864699147237</v>
+      </c>
+      <c r="G7">
+        <v>5.384030920762236</v>
+      </c>
+      <c r="H7">
+        <v>4.416744640490035</v>
+      </c>
+      <c r="I7">
+        <v>3.086546994775801</v>
+      </c>
+      <c r="J7">
+        <v>2031</v>
+      </c>
+      <c r="K7">
+        <v>66.1055769483837</v>
+      </c>
+      <c r="L7">
+        <v>2030</v>
+      </c>
+      <c r="M7">
+        <v>66.1055769483837</v>
+      </c>
+      <c r="N7">
+        <v>64.54108721207183</v>
+      </c>
+      <c r="O7">
+        <v>62.83457706423353</v>
+      </c>
+      <c r="Q7">
+        <v>3.520290648629189</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17">
+      <c r="A8" t="s">
+        <v>154</v>
+      </c>
+      <c r="B8">
+        <v>1.55</v>
+      </c>
+      <c r="C8">
+        <v>0.3876378678126633</v>
+      </c>
+      <c r="D8" t="s">
+        <v>196</v>
+      </c>
+      <c r="E8">
+        <v>8.548271921289457</v>
+      </c>
+      <c r="F8">
+        <v>37.30793225743088</v>
+      </c>
+      <c r="G8">
+        <v>5.785256966062674</v>
+      </c>
+      <c r="H8">
+        <v>6.061215470501122</v>
+      </c>
+      <c r="I8">
+        <v>6.486601199839658</v>
+      </c>
+      <c r="K8">
+        <v>108.6969482402365</v>
+      </c>
+      <c r="L8">
+        <v>2040</v>
+      </c>
+      <c r="M8">
+        <v>74.07533385152752</v>
+      </c>
+      <c r="N8">
+        <v>91.2706933000166</v>
+      </c>
+      <c r="O8">
+        <v>108.6969482402365</v>
+      </c>
+      <c r="Q8">
+        <v>4.758550641184393</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17">
+      <c r="A9" t="s">
+        <v>155</v>
+      </c>
+      <c r="B9">
+        <v>1.55</v>
+      </c>
+      <c r="C9">
+        <v>0.3876378678126633</v>
+      </c>
+      <c r="D9" t="s">
+        <v>196</v>
+      </c>
+      <c r="E9">
+        <v>8.548271921289457</v>
+      </c>
+      <c r="F9">
+        <v>37.30793225743088</v>
+      </c>
+      <c r="G9">
+        <v>5.485256966062674</v>
+      </c>
+      <c r="H9">
+        <v>4.535966877109199</v>
+      </c>
+      <c r="I9">
+        <v>3.244189921853434</v>
+      </c>
+      <c r="J9">
+        <v>2031</v>
+      </c>
+      <c r="K9">
+        <v>66.70552558077179</v>
+      </c>
+      <c r="L9">
+        <v>2031</v>
+      </c>
+      <c r="M9">
+        <v>66.60000598167082</v>
+      </c>
+      <c r="N9">
+        <v>65.77043644979558</v>
+      </c>
+      <c r="O9">
+        <v>64.83203327525396</v>
+      </c>
+      <c r="Q9">
+        <v>3.578786255115994</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17">
+      <c r="A10" t="s">
+        <v>154</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>0.287</v>
+      </c>
+      <c r="D10" t="s">
+        <v>197</v>
+      </c>
+      <c r="E10">
+        <v>6.324511209781276</v>
+      </c>
+      <c r="F10">
+        <v>27.61288908976673</v>
+      </c>
+      <c r="G10">
+        <v>5.711194154467356</v>
+      </c>
+      <c r="H10">
+        <v>5.973981438017038</v>
+      </c>
+      <c r="I10">
+        <v>6.371169406434555</v>
+      </c>
+      <c r="K10">
+        <v>107.2336747399897</v>
+      </c>
+      <c r="L10">
+        <v>2040</v>
+      </c>
+      <c r="M10">
+        <v>73.71194808935667</v>
+      </c>
+      <c r="N10">
+        <v>90.36949971487616</v>
+      </c>
+      <c r="O10">
+        <v>107.2336747399897</v>
+      </c>
+      <c r="Q10">
+        <v>4.715659105537023</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17">
+      <c r="A11" t="s">
+        <v>155</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11">
+        <v>0.287</v>
+      </c>
+      <c r="D11" t="s">
+        <v>197</v>
+      </c>
+      <c r="E11">
+        <v>6.324511209781276</v>
+      </c>
+      <c r="F11">
+        <v>27.61288908976673</v>
+      </c>
+      <c r="G11">
+        <v>5.411194154467356</v>
+      </c>
+      <c r="H11">
+        <v>4.448736871454138</v>
+      </c>
+      <c r="I11">
+        <v>3.128847311158677</v>
+      </c>
+      <c r="J11">
+        <v>2031</v>
+      </c>
+      <c r="K11">
+        <v>66.23822052220449</v>
+      </c>
+      <c r="L11">
+        <v>2031</v>
+      </c>
+      <c r="M11">
+        <v>66.23820415131104</v>
+      </c>
+      <c r="N11">
+        <v>64.87092592274449</v>
+      </c>
+      <c r="O11">
+        <v>63.37053319227711</v>
+      </c>
+      <c r="Q11">
+        <v>3.535984893012419</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17">
+      <c r="A12" t="s">
+        <v>154</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12">
+        <v>0.5370889469759117</v>
+      </c>
+      <c r="D12" t="s">
+        <v>198</v>
+      </c>
+      <c r="E12">
+        <v>11.85643014786837</v>
+      </c>
+      <c r="F12">
+        <v>51.71733780312103</v>
+      </c>
+      <c r="G12">
+        <v>5.895249381915646</v>
+      </c>
+      <c r="H12">
+        <v>6.190770222805426</v>
+      </c>
+      <c r="I12">
+        <v>6.658051476937715</v>
+      </c>
+      <c r="K12">
+        <v>110.8705549601242</v>
+      </c>
+      <c r="L12">
+        <v>2040</v>
+      </c>
+      <c r="M12">
+        <v>74.6155022490132</v>
+      </c>
+      <c r="N12">
+        <v>92.6095598240873</v>
+      </c>
+      <c r="O12">
+        <v>110.8705549601242</v>
+      </c>
+      <c r="Q12">
+        <v>4.822276193136064</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17">
+      <c r="A13" t="s">
+        <v>155</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13">
+        <v>0.5370889469759117</v>
+      </c>
+      <c r="D13" t="s">
+        <v>198</v>
+      </c>
+      <c r="E13">
+        <v>11.85643014786837</v>
+      </c>
+      <c r="F13">
+        <v>51.71733780312103</v>
+      </c>
+      <c r="G13">
+        <v>5.595249381915645</v>
+      </c>
+      <c r="H13">
+        <v>4.665515645892417</v>
+      </c>
+      <c r="I13">
+        <v>3.4155076516056</v>
+      </c>
+      <c r="J13">
+        <v>2032</v>
+      </c>
+      <c r="K13">
+        <v>67.48084364411615</v>
+      </c>
+      <c r="L13">
+        <v>2032</v>
+      </c>
+      <c r="M13">
+        <v>67.13782026862528</v>
+      </c>
+      <c r="N13">
+        <v>67.10680153741228</v>
+      </c>
+      <c r="O13">
+        <v>67.00300426281882</v>
+      </c>
+      <c r="Q13">
+        <v>3.642377787100643</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17">
+      <c r="A14" t="s">
+        <v>154</v>
+      </c>
+      <c r="B14">
+        <v>1.55</v>
+      </c>
+      <c r="C14">
+        <v>0.6746378678126632</v>
+      </c>
+      <c r="D14" t="s">
+        <v>198</v>
+      </c>
+      <c r="E14">
+        <v>14.90724334233834</v>
+      </c>
+      <c r="F14">
+        <v>64.99172541765893</v>
+      </c>
+      <c r="G14">
+        <v>5.996488741389228</v>
+      </c>
+      <c r="H14">
+        <v>6.310016713258292</v>
+      </c>
+      <c r="I14">
+        <v>6.815878952205352</v>
+      </c>
+      <c r="K14">
+        <v>112.8716809513749</v>
+      </c>
+      <c r="L14">
+        <v>2040</v>
+      </c>
+      <c r="M14">
+        <v>75.11320895515519</v>
+      </c>
+      <c r="N14">
+        <v>93.84239185934949</v>
+      </c>
+      <c r="O14">
+        <v>112.8716809513749</v>
+      </c>
+      <c r="Q14">
+        <v>4.880958398171277</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17">
+      <c r="A15" t="s">
+        <v>155</v>
+      </c>
+      <c r="B15">
+        <v>1.55</v>
+      </c>
+      <c r="C15">
+        <v>0.6746378678126632</v>
+      </c>
+      <c r="D15" t="s">
+        <v>198</v>
+      </c>
+      <c r="E15">
+        <v>14.90724334233834</v>
+      </c>
+      <c r="F15">
+        <v>64.99172541765893</v>
+      </c>
+      <c r="G15">
+        <v>5.696488741389229</v>
+      </c>
+      <c r="H15">
+        <v>4.784756625619105</v>
+      </c>
+      <c r="I15">
+        <v>3.573213021689391</v>
+      </c>
+      <c r="K15">
+        <v>69.00170216637231</v>
+      </c>
+      <c r="L15">
+        <v>2040</v>
+      </c>
+      <c r="M15">
+        <v>67.6333583225224</v>
+      </c>
+      <c r="N15">
+        <v>68.33732920093439</v>
+      </c>
+      <c r="O15">
+        <v>69.00170216637231</v>
+      </c>
+      <c r="Q15">
+        <v>3.700936530344884</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H16"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B1" t="s">
+        <v>200</v>
+      </c>
+      <c r="C1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D1" t="s">
+        <v>202</v>
+      </c>
+      <c r="E1" t="s">
+        <v>203</v>
+      </c>
+      <c r="F1" t="s">
+        <v>204</v>
+      </c>
+      <c r="G1" t="s">
+        <v>205</v>
+      </c>
+      <c r="H1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2">
+        <v>2026</v>
+      </c>
+      <c r="B2">
+        <v>62.58890458136189</v>
+      </c>
+      <c r="C2">
+        <v>62.58890458136189</v>
+      </c>
+      <c r="D2">
+        <v>62.58890458136189</v>
+      </c>
+      <c r="E2">
+        <v>62.58890458136189</v>
+      </c>
+      <c r="F2">
+        <v>62.58890458136189</v>
+      </c>
+      <c r="G2">
+        <v>62.58890458136189</v>
+      </c>
+      <c r="H2">
+        <v>62.58890458136189</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3">
+        <v>2027</v>
+      </c>
+      <c r="B3">
+        <v>64.93452689744312</v>
+      </c>
+      <c r="C3">
+        <v>64.40087608453982</v>
+      </c>
+      <c r="D3">
+        <v>65.11927783670889</v>
+      </c>
+      <c r="E3">
+        <v>64.40087608453982</v>
+      </c>
+      <c r="F3">
+        <v>64.23452689744312</v>
+      </c>
+      <c r="G3">
+        <v>63.3477288453457</v>
+      </c>
+      <c r="H3">
+        <v>64.70087608453981</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4">
+        <v>2028</v>
+      </c>
+      <c r="B4">
+        <v>67.58446344622884</v>
+      </c>
+      <c r="C4">
+        <v>65.30601807575621</v>
+      </c>
+      <c r="D4">
+        <v>67.61679648032644</v>
+      </c>
+      <c r="E4">
+        <v>71.6510009632115</v>
+      </c>
+      <c r="F4">
+        <v>65.0806910989761</v>
+      </c>
+      <c r="G4">
+        <v>63.46791745915831</v>
+      </c>
+      <c r="H4">
+        <v>65.89066956712199</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5">
+        <v>2029</v>
+      </c>
+      <c r="B5">
+        <v>70.49357005145103</v>
+      </c>
+      <c r="C5">
+        <v>65.36001635459498</v>
+      </c>
+      <c r="D5">
+        <v>69.89307888062643</v>
+      </c>
+      <c r="E5">
+        <v>74.05769779985735</v>
+      </c>
+      <c r="F5">
+        <v>65.16723239559157</v>
+      </c>
+      <c r="G5">
+        <v>62.95181813709121</v>
+      </c>
+      <c r="H5">
+        <v>66.21650329616409</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6">
+        <v>2030</v>
+      </c>
+      <c r="B6">
+        <v>73.62563007426643</v>
+      </c>
+      <c r="C6">
+        <v>65.20797390976422</v>
+      </c>
+      <c r="D6">
+        <v>71.6678292693645</v>
+      </c>
+      <c r="E6">
+        <v>74.64756096677065</v>
+      </c>
+      <c r="F6">
+        <v>64.53642381027402</v>
+      </c>
+      <c r="G6">
+        <v>61.56590024996358</v>
+      </c>
+      <c r="H6">
+        <v>66.32577686766911</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7">
+        <v>2031</v>
+      </c>
+      <c r="B7">
+        <v>76.91571689680475</v>
+      </c>
+      <c r="C7">
+        <v>64.9071361732591</v>
+      </c>
+      <c r="D7">
+        <v>72.91047367921412</v>
+      </c>
+      <c r="E7">
+        <v>74.99032613545374</v>
+      </c>
+      <c r="F7">
+        <v>64.00428277085403</v>
+      </c>
+      <c r="G7">
+        <v>60.10105472545386</v>
+      </c>
+      <c r="H7">
+        <v>66.27692683268637</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8">
+        <v>2032</v>
+      </c>
+      <c r="B8">
+        <v>80.19217073544627</v>
+      </c>
+      <c r="C8">
+        <v>64.41922013381722</v>
+      </c>
+      <c r="D8">
+        <v>73.57912643541387</v>
+      </c>
+      <c r="E8">
+        <v>75.0456458856188</v>
+      </c>
+      <c r="F8">
+        <v>63.41682447393597</v>
+      </c>
+      <c r="G8">
+        <v>58.56496087171271</v>
+      </c>
+      <c r="H8">
+        <v>66.03017502301574</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9">
+        <v>2033</v>
+      </c>
+      <c r="B9">
+        <v>83.46194582525446</v>
+      </c>
+      <c r="C9">
+        <v>63.75226124997421</v>
+      </c>
+      <c r="D9">
+        <v>73.88919028036351</v>
+      </c>
+      <c r="E9">
+        <v>74.83962172719177</v>
+      </c>
+      <c r="F9">
+        <v>62.78373296494627</v>
+      </c>
+      <c r="G9">
+        <v>56.9756007575451</v>
+      </c>
+      <c r="H9">
+        <v>65.59402179107478</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10">
+        <v>2034</v>
+      </c>
+      <c r="B10">
+        <v>86.73106913700117</v>
+      </c>
+      <c r="C10">
+        <v>63.0139498381896</v>
+      </c>
+      <c r="D10">
+        <v>73.94867584698677</v>
+      </c>
+      <c r="E10">
+        <v>74.49526406304325</v>
+      </c>
+      <c r="F10">
+        <v>62.11274998717341</v>
+      </c>
+      <c r="G10">
+        <v>55.34721584948421</v>
+      </c>
+      <c r="H10">
+        <v>65.07660237890576</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11">
+        <v>2035</v>
+      </c>
+      <c r="B11">
+        <v>90.00473769204891</v>
+      </c>
+      <c r="C11">
+        <v>62.30735065942545</v>
+      </c>
+      <c r="D11">
+        <v>73.8623589199684</v>
+      </c>
+      <c r="E11">
+        <v>74.12875101713996</v>
+      </c>
+      <c r="F11">
+        <v>61.41004603265997</v>
+      </c>
+      <c r="G11">
+        <v>53.69103706293036</v>
+      </c>
+      <c r="H11">
+        <v>64.58140736244037</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12">
+        <v>2036</v>
+      </c>
+      <c r="B12">
+        <v>93.28741693369645</v>
+      </c>
+      <c r="C12">
+        <v>61.63110159776822</v>
+      </c>
+      <c r="D12">
+        <v>73.73198829228667</v>
+      </c>
+      <c r="E12">
+        <v>73.74969255356471</v>
+      </c>
+      <c r="F12">
+        <v>60.6805260430722</v>
+      </c>
+      <c r="G12">
+        <v>52.01588866560481</v>
+      </c>
+      <c r="H12">
+        <v>64.10748215096793</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13">
+        <v>2037</v>
+      </c>
+      <c r="B13">
+        <v>96.58293494872801</v>
+      </c>
+      <c r="C13">
+        <v>60.98389904342599</v>
+      </c>
+      <c r="D13">
+        <v>73.55642246441616</v>
+      </c>
+      <c r="E13">
+        <v>73.36562480500363</v>
+      </c>
+      <c r="F13">
+        <v>59.92807915176644</v>
+      </c>
+      <c r="G13">
+        <v>50.32868136290389</v>
+      </c>
+      <c r="H13">
+        <v>63.65391315572158</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14">
+        <v>2038</v>
+      </c>
+      <c r="B14">
+        <v>99.89456963935189</v>
+      </c>
+      <c r="C14">
+        <v>60.36449537975121</v>
+      </c>
+      <c r="D14">
+        <v>73.33513102609251</v>
+      </c>
+      <c r="E14">
+        <v>72.98240193531805</v>
+      </c>
+      <c r="F14">
+        <v>59.15578138347605</v>
+      </c>
+      <c r="G14">
+        <v>48.63481092680315</v>
+      </c>
+      <c r="H14">
+        <v>63.21982602874725</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15">
+        <v>2039</v>
+      </c>
+      <c r="B15">
+        <v>103.2251274661083</v>
+      </c>
+      <c r="C15">
+        <v>59.7716965782019</v>
+      </c>
+      <c r="D15">
+        <v>73.16805726026966</v>
+      </c>
+      <c r="E15">
+        <v>72.60452330653708</v>
+      </c>
+      <c r="F15">
+        <v>58.36605933674945</v>
+      </c>
+      <c r="G15">
+        <v>46.93847799930541</v>
+      </c>
+      <c r="H15">
+        <v>62.80438397741724</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16">
+        <v>2040</v>
+      </c>
+      <c r="B16">
+        <v>106.5770133547019</v>
+      </c>
+      <c r="C16">
+        <v>59.20435989660484</v>
+      </c>
+      <c r="D16">
+        <v>73.05212746939111</v>
+      </c>
+      <c r="E16">
+        <v>72.23540329299968</v>
+      </c>
+      <c r="F16">
+        <v>57.56082183010944</v>
+      </c>
+      <c r="G16">
+        <v>45.24294311860554</v>
+      </c>
+      <c r="H16">
+        <v>62.4067861513396</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>